<commit_message>
feat(population): per-capita in map tooltips
</commit_message>
<xml_diff>
--- a/config/regions.xlsx
+++ b/config/regions.xlsx
@@ -1,29 +1,30 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jonas\Documents\Hector\Kooperationsphase IO-Modelle\exiobase_explorer\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F7FEF61-765E-4B4D-B246-E3448DB1027F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC1853F7-5E5A-45EA-A658-3E9800646ACF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Exiobase" sheetId="1" r:id="rId1"/>
     <sheet name="map" sheetId="4" r:id="rId2"/>
     <sheet name="Deutsch" sheetId="2" r:id="rId3"/>
     <sheet name="Englisch" sheetId="3" r:id="rId4"/>
+    <sheet name="population" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="608" uniqueCount="298">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="659" uniqueCount="299">
   <si>
     <t>region</t>
   </si>
@@ -917,6 +918,9 @@
   </si>
   <si>
     <t>continent</t>
+  </si>
+  <si>
+    <t>population</t>
   </si>
 </sst>
 </file>
@@ -3832,4 +3836,267 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{54130B71-89B3-47B7-9AD0-D3A95FB56FB2}">
+  <dimension ref="A1:B50"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A10" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A11" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A12" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A13" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A14" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A15" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A16" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A17" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A18" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A19" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A20" s="2" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A21" s="2" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A22" s="2" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A23" s="2" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A24" s="2" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A25" s="2" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A26" s="2" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A27" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A28" s="2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A29" s="2" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="30" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A30" s="2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="31" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A31" s="2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="32" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A32" s="2" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A33" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A34" s="2" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="35" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A35" s="2" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="36" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A36" s="2" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="37" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A37" s="2" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="38" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A38" s="2" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="39" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A39" s="2" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="40" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A40" s="2" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="41" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A41" s="2" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="42" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A42" s="2" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="43" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A43" s="2" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="44" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A44" s="2" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="45" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A45" s="2" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="46" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A46" s="2" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="47" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A47" s="2" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="48" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A48" s="2" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="49" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A49" s="2" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="50" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A50" s="2" t="s">
+        <v>49</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Update population sheet in regions.xlsx
</commit_message>
<xml_diff>
--- a/config/regions.xlsx
+++ b/config/regions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jonas\Documents\Hector\Kooperationsphase IO-Modelle\exiobase_explorer\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC1853F7-5E5A-45EA-A658-3E9800646ACF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8669A5A5-06D0-44C9-BBE9-D1E89C9DD7A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3855,245 +3855,392 @@
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
+      <c r="B2" s="2">
+        <v>9120000</v>
+      </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>2</v>
       </c>
+      <c r="B3" s="2">
+        <v>11820000</v>
+      </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>3</v>
       </c>
+      <c r="B4" s="2">
+        <v>6450000</v>
+      </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>4</v>
       </c>
+      <c r="B5" s="2">
+        <v>1360000</v>
+      </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>5</v>
       </c>
+      <c r="B6" s="2">
+        <v>10740000</v>
+      </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>6</v>
       </c>
+      <c r="B7" s="2">
+        <v>84550000</v>
+      </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>7</v>
       </c>
+      <c r="B8" s="2">
+        <v>5980000</v>
+      </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>8</v>
       </c>
+      <c r="B9" s="2">
+        <v>1370000</v>
+      </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>9</v>
       </c>
+      <c r="B10" s="2">
+        <v>47890000</v>
+      </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>10</v>
       </c>
+      <c r="B11" s="2">
+        <v>5620000</v>
+      </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>11</v>
       </c>
+      <c r="B12" s="2">
+        <v>66550000</v>
+      </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>12</v>
       </c>
+      <c r="B13" s="2">
+        <v>9940000</v>
+      </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>13</v>
       </c>
+      <c r="B14" s="2">
+        <v>3860000</v>
+      </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>14</v>
       </c>
+      <c r="B15" s="2">
+        <v>9590000</v>
+      </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B16" s="2">
+        <v>5310000</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B17" s="2">
+        <v>58760000</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B18" s="2">
+        <v>2850000</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B19" s="2">
+        <v>681000</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B20" s="2">
+        <v>1870000</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B21" s="2">
+        <v>545000</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B22" s="2">
+        <v>18230000</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B23" s="2">
+        <v>37560000</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B24" s="2">
+        <v>10430000</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B25" s="2">
+        <v>19020000</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B26" s="2">
+        <v>10610000</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B27" s="2">
+        <v>2120000</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B28" s="2">
+        <v>5420000</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B29" s="2">
+        <v>69550000</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="31" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B30" s="2">
+        <v>345427000</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="32" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B31" s="2">
+        <v>123104000</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B32" s="2">
+        <v>1408281000</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B33" s="2">
+        <v>40127000</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="35" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B34" s="2">
+        <v>51718000</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="36" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B35" s="2">
+        <v>211999000</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="37" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B36" s="2">
+        <v>1463866000</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="38" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B37" s="2">
+        <v>131947000</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="39" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B38" s="2">
+        <v>143997000</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="40" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B39" s="2">
+        <v>26974000</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="41" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B40" s="2">
+        <v>8922000</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="42" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B41" s="2">
+        <v>87686000</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="43" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B42" s="2">
+        <v>23420000</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A43" s="2" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="44" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B43" s="2">
+        <v>5576000</v>
+      </c>
+    </row>
+    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A44" s="2" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="45" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B44" s="2">
+        <v>281190000</v>
+      </c>
+    </row>
+    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A45" s="2" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="46" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B45" s="2">
+        <v>63212000</v>
+      </c>
+    </row>
+    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A46" s="2" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="47" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B46" s="2">
+        <v>876300000</v>
+      </c>
+    </row>
+    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A47" s="2" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="48" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B47" s="2">
+        <v>449800000</v>
+      </c>
+    </row>
+    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A48" s="2" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="49" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B48" s="2">
+        <v>92900000</v>
+      </c>
+    </row>
+    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A49" s="2" t="s">
         <v>48</v>
       </c>
-    </row>
-    <row r="50" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B49" s="2">
+        <v>1444900000</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A50" s="2" t="s">
         <v>49</v>
+      </c>
+      <c r="B50" s="2">
+        <v>293874618</v>
       </c>
     </row>
   </sheetData>

</xml_diff>